<commit_message>
Buffalo Wabs 2026-08-28: Rev 2.1 rebuild (17 ch) recovered from stash
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audio/Fountain Square/2026-08-28 Buffalo Wabs and the Price Hill Hustle/Buffalo Wabs and the Price Hill Hustle - Input List.xlsx
+++ b/audio/Fountain Square/2026-08-28 Buffalo Wabs and the Price Hill Hustle/Buffalo Wabs and the Price Hill Hustle - Input List.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fountain Square (outdoor) · 2026-08-28 · Rev 1.0 Deep Think</t>
+          <t>Fountain Square (outdoor) · 2026-08-28 · Rev 2.1 Deep Think</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mandolin</t>
+          <t>Acoustic Mandolin</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Onboard pickup, XLR line feed (locker-exempt). Confirm phantom need at line check.</t>
+          <t>Scott's acoustic mandolin, onboard pickup XLR (locker-exempt). Confirm phantom need at line check.</t>
         </is>
       </c>
     </row>
@@ -785,12 +785,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Electric Mandolin</t>
+          <t>Resonator / Dobro</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>XLR (DI)</t>
+          <t>XLR (pickup DI)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Electric mandolin, XLR (locker-exempt). Warmer/fuller than the acoustic mando — lighter piezo character.</t>
+          <t>Reso/dobro onboard pickup, XLR (locker-exempt).</t>
         </is>
       </c>
     </row>
@@ -815,12 +815,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Resonator / Dobro</t>
+          <t>Electric Mandolin / Electric Guitar</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>XLR (pickup DI)</t>
+          <t>XLR (cab-sim direct)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Reso/dobro onboard pickup, XLR (locker-exempt).</t>
+          <t>SHARED channel — electric mandolin OR Matt's electric guitar (XLR, cab-sim/modeler direct feed). Not simultaneous. RETUNE at soundcheck for the active instrument: electric guitar wants the LPF for fizz + more 3.5k trim; electric mando wants a hair more 1.5k. Locker-exempt (line feed).</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tenor Banjo</t>
+          <t>Acoustic Guitar</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Tenor banjo onboard pickup, XLR (locker-exempt). Feedback-prone outdoors at level.</t>
+          <t>Matt's acoustic, onboard pickup XLR (locker-exempt).</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Acoustic Guitar</t>
+          <t>Doubling (Scott)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -895,47 +895,47 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Matt's acoustic, onboard pickup XLR (locker-exempt).</t>
+          <t>Utility instrument-swap channel — mandolin / 5-string banjo / acoustic guitar. This is where the 5-string banjo now lives (the dedicated banjo channel was dropped in this rev). RETUNE the 2.5k quack cut per whichever instrument is live: banjo wants it narrower + a 250 boom cut, acoustic a hair lower.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Doubling (Scott)</t>
+          <t>Vocal (harmony)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>XLR (pickup DI)</t>
+          <t>Shure Beta 58A (wireless)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Local 18</t>
+          <t>Local 33</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>DI</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Utility instrument-swap channel (mandolin / 5-string banjo / acoustic). RETUNE the 2.5k quack cut per whichever instrument is live at soundcheck — banjo wants it narrower, acoustic a hair lower.</t>
+          <t>House wireless 1 (FSQ fader 33). Overrides the template's stock wireless curve/notch — ring out at soundcheck. COMP (doc only): Blue/Neve ~2.5:1, 3–4 dB GR.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Vocal (harmony)</t>
+          <t>LEAD Vocal (Matt)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Local 33</t>
+          <t>Local 34</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -955,17 +955,17 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>House wireless 1 (FSQ fader 33). Overrides the template's stock wireless curve/notch — ring out at soundcheck. COMP (doc only): Blue/Neve ~2.5:1, 3–4 dB GR.</t>
+          <t>House wireless 2 (FSQ fader 34) — Matt 'Buffalo Wabs', LEAD. Overrides template wireless curve — most body kept of the four. COMP (doc only): Blue/Neve ~3:1, 3–4 dB GR.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LEAD Vocal (Matt)</t>
+          <t>Vocal (drummer, at kit)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Local 34</t>
+          <t>Local 35</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -985,17 +985,17 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>House wireless 2 (FSQ fader 34) — Matt 'Buffalo Wabs', LEAD. Overrides template wireless curve — most body kept of the four. COMP (doc only): Blue/Neve ~3:1, 3–4 dB GR.</t>
+          <t>House wireless 3 (FSQ fader 35) — Casey sings FROM THE KIT, so kit bleed into this mic is the constraint. Ride the digital trim; the supercardioid pattern is doing the rejection. GATE/DUCK (doc only): consider a shallow duck off the kit VCA. COMP (doc only): Blue/Neve ~3:1, 3–4 dB GR.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Vocal (drummer, at kit)</t>
+          <t>Vocal (bass, low)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Local 35</t>
+          <t>Local 36</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1014,36 +1014,6 @@
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>House wireless 3 (FSQ fader 35) — Casey sings FROM THE KIT, so kit bleed into this mic is the constraint. Ride the digital trim; the supercardioid pattern is doing the rejection. GATE/DUCK (doc only): consider a shallow duck off the kit VCA. COMP (doc only): Blue/Neve ~3:1, 3–4 dB GR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>36</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Vocal (bass, low)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Shure Beta 58A (wireless)</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Local 36</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>House wireless 4 (FSQ fader 36) — Bill 'Bullseye Bill', the upright player; treated as the low/bass voice of the harmony stack. Lowest HPF of the four. COMP (doc only): Blue/Neve ~2.5:1, 3–4 dB GR.</t>
         </is>
@@ -1060,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1105,22 +1075,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Plates 1 / #06 Vocal Plate</t>
+          <t>Seventh Heaven Pro — Plates 1 / #06 Vocal Plate</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Decay 1.5s (factory) · PreDelay 24ms (factory) · VLF −19 (factory) · E/L Max Early · Late −6 (raised from the factory reference — outdoors carries the late field) · Late Rolloff 6400 (factory)</t>
+          <t>Decay 1.5s (factory) · PreDelay 24ms (factory) · VLF -19 (factory) · E/L Max Early · Late -6 (raised from the factory reference for outdoors) · Late Rolloff 6400 (factory)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Return LC 160 Hz; ducker Reverb mode, Thr −22 dB, Rel ~250 ms</t>
+          <t>Return-channel EQ (Q225): HPF 200 · LPF 9k · B3 -3 @ 3.5k Q2 · B2 -3 @ 500 Q1.8</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>The harmony-ballad + lead workhorse. Plate sheen sits the four-part harmony forward with no room outdoors to muddy it — the big-moment ballad throw.</t>
+          <t>Lead + harmony-ballad plate. Its tail already rolls at 6.4k with a clean low (VLF -19), so it needs the least top-taming — LPF stays at 9k to keep the sheen that lifts the harmony; -3@3.5k stops it going strident when all four voices stack, -3@500 clears the dense-plate low-mid.</t>
         </is>
       </c>
     </row>
@@ -1132,22 +1102,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chambers 1 / #10 Vocal Chamber</t>
+          <t>Waves CLA Epic — The Vocal 3 preset (plate + slap)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Decay 1.6s (factory) · PreDelay 0 (factory) · VLF −10 (factory) · E/L Max Early · Late −8 (near factory ref) · Late Rolloff 8000 (factory)</t>
+          <t>CLA Epic lead-vocal preset (Chris Lord-Alge plate + slap/throw). Keep the preset plate time/pre-delay; set HF Damp so the slap repeats do not spit. Bright, forward lead verb.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Return LC 150 Hz; ducker Reverb mode, Thr −22 dB</t>
+          <t>Return-channel EQ (Q225): HPF 220 · LPF 7.5k · B3 -4 @ 4k Q2 · B2 -3 @ 450 Q1.8</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Warmer, more natural than the plate — flatters a roots baritone lead on mid-tempo numbers. Hands off with the Vocal Plate song to song.</t>
+          <t>The brightest, most forward return in the set. Gets the hardest top pull (LPF 7.5k) and deepest de-harsh (-4@4k) or it turns edgy/sibilant outdoors in the humidity and the slap repeats spit; HPF 220 keeps those repeats articulate. Ring this one out at soundcheck — most feedback-prone.</t>
         </is>
       </c>
     </row>
@@ -1159,22 +1129,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rooms 1 / #27 Small Room</t>
+          <t>Soundtoys EchoBoy Hallway (30% wet) → Seventh Heaven Pro — Chambers 1 / #17 Sunset Chamber</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Decay 0.6s (factory) · PreDelay 0 (factory) · VLF −12 (factory) · E/L Max Early · Late −10 · Late Rolloff 6800 (factory)</t>
+          <t>Serial chain: EchoBoy Hallway at 30% wet feeding Sunset Chamber (Decay 2.15s factory · PreDelay 20ms factory · VLF -20 factory · E/L Max Early · Late -8 · Late Rolloff 7200 factory). Warm, dark, long — the big-moment/ballad return.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Return LC 200 Hz</t>
+          <t>Return-channel EQ (Q225): HPF 260 · LPF 10k · B3 -2 @ 3k Q2 · B2 -4 @ 350 Q1.6</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>The dry option for the fast foot-stompers — a short tail keeps consonants crisp in the open air so the lyric survives the tempo.</t>
+          <t>Warm/dark and LONG (2.15s) with EchoBoy tape warmth ahead of it — already soft up top, so LPF stays gentle at 10k and the 3k cut is only -2 (over-darkening kills the bloom). The work is down low: highest HPF (260) + deepest mud cut (-4@350), because a long tail plus a serial tape stage is where this chain turns to soup on a busy number.</t>
         </is>
       </c>
     </row>
@@ -1186,91 +1156,64 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rooms 1 / #36 Long Wood Room</t>
+          <t>Waves CLA Epic — Acoustic Guitar Room 1 preset</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Decay 1.2s (factory) · PreDelay 0 (factory) · VLF −9 (factory) · E/L Max Early · Late −8 · Late Rolloff 7600 (factory)</t>
+          <t>CLA Epic room voiced for acoustic guitar — tight, present room. Glue for the acoustic pickers (mando/reso/banjo/acoustic). Keep the preset time short.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Return LC 200 Hz, HS −2 @ 8 k</t>
+          <t>Return-channel EQ (Q225): HPF 180 · LPF 8k · B3 -4 @ 2.5k Q2 · B2 -3 @ 400 Q1.8</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Wood-room glue for the acoustic pickers (mando/reso/banjo/acoustic) — the woody character matches the instruments and cohere them outdoors without the artificial sheen a plate would put on a banjo.</t>
+          <t>Key move: -4@2.5k is the exact piezo-quack/metallic zone cut on every string source, so this room tail cannot re-energize what the channel EQ removed. CLA brightness plus banjo/reso metallic top is why LPF sits at 8k; HPF 180 lets a little instrument body bloom while blocking mud.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>instrument</t>
+          <t>drum</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chambers 1 / #09 Snare Chamber</t>
+          <t>Waves Atlas Reverb — Big Drum Room preset</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Decay 1.2s (factory) · PreDelay 10ms (factory) · VLF −19 (factory) · E/L Max Early · Late −10 · Late Rolloff 5600 (factory)</t>
+          <t>Atlas algorithmic large drum room. Big body + cymbal wash; consider trimming the program decay for the open-air mix.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Return LC 250 Hz</t>
+          <t>Return-channel EQ (Q225): HPF 160 · LPF 8k · B3 -3 @ 3k Q2 · B2 -4 @ 300 Q1.8</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>A short snare splash for the big backbeats on the foot-stompers — snap without mud. Ride it up only on the uptempo numbers, off under the ballads.</t>
+          <t>A big room signature problem is low-mid body and cymbal wash, both amplified by the size — HPF 160 keeps kick/floor tom out so punch stays dry, -4@300 carves the boxy room resonance a big algorithm piles up, -3@3k tames cymbal/hat wash before it smears the outdoor mix. Cuts-only — no snap boost outdoors.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ambiences 1 / #01 Large Ambience</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Decay 0.8s (factory) · PreDelay 10ms (factory) · VLF −10 (factory) · E/L Max Early · Late −10 · Late Rolloff 6000 (factory)</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+          <t>TOGETHER</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>A whisper of overall air so the open-air stage isn't bone-dry — no audible tail, just glue under the whole band when a number wants it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TOGETHER</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Two lead vocal returns hand off song to song: Vocal Plate is the default forward lead + the ballad harmony bed; Vocal Chamber is the warmer mid-tempo option; on the fast foot-stompers ride the dry Small Room instead so the lyric stays articulate outdoors. Long Wood Room is the acoustic-instrument glue — mandolin, resonator, banjo, acoustic guitar feed it as a group for cohesion; keep the upright out of it. Snare Chamber is a backbeat-only splash on uptempo numbers, off under ballads. Large Ambience is a whisper of overall band air, ridden up only when a number feels bone-dry. All returns 100% wet, level ridden by the sends.</t>
+          <t>Five real returns. Three vocal returns hand off by song type: the Seventh Heaven Vocal Plate is the default forward lead + harmony bed; the CLA Epic Vocal 3 (bright plate+slap) is the up-front, aggressive option for a feature or a driving number; the EchoBoy-&gt;Sunset Chamber chain is the warm, long big-moment/ballad wash — ride it up only on the slow, spacious tunes and pull it under fast ones. The CLA Epic Acoustic Guitar Room glues the acoustic pickers (mandolin/resonator/banjo/acoustic) as a group; keep the upright out of it. The Atlas Big Drum Room sits under the kit — ride it up on the foot-stompers, off under ballads. All returns 100% wet, level ridden by the sends; return EQ per the plugin_eq lines (Q225 return-channel or the plugin own filter — same targets).</t>
         </is>
       </c>
     </row>

</xml_diff>